<commit_message>
added more spec WIP
</commit_message>
<xml_diff>
--- a/docs/spec/ARM.xlsx
+++ b/docs/spec/ARM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EitanKrimer\Documents\university\ADSS\ADSS_Group_Y\docs\spec\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E98275-9B86-4231-8B76-9911F0432A3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBB33EFA-9F31-449B-B084-A44D2B0EBB48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ARM" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="52">
   <si>
     <t>ID</t>
   </si>
@@ -950,12 +950,662 @@
 - OPTIONAL Recroded weight at site</t>
     </r>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to start a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to create a future </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to update a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to delete a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> a transport manager to create a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="7" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>driver</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to edit a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="7" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>driver</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to delete a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="7" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>driver</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to create a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>truck</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to edit a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>truck</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to delete a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>truck</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>admin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to create a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>branch</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>admin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to edit a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>branch</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>admin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to delete a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>branch</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1112,13 +1762,43 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF00B050"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="7" tint="-0.249977111117893"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="7">
@@ -1211,7 +1891,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -1220,9 +1900,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1236,6 +1913,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -1258,8 +1938,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1549,7 +2232,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="21" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
@@ -1604,11 +2287,11 @@
       <c r="C3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
       <c r="G3" s="3" t="s">
         <v>15</v>
       </c>
@@ -1624,7 +2307,7 @@
       <c r="C4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>35</v>
       </c>
       <c r="E4" s="3" t="s">
@@ -1648,7 +2331,7 @@
       <c r="C5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E5" s="3" t="s">
@@ -1663,7 +2346,7 @@
     </row>
     <row r="6" spans="1:7" ht="141.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
-        <f t="shared" ref="A6:A18" si="0">A5+1</f>
+        <f t="shared" ref="A6:A31" si="0">A5+1</f>
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -1672,7 +2355,7 @@
       <c r="C6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E6" s="3" t="s">
@@ -1696,7 +2379,7 @@
       <c r="C7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="5" t="s">
         <v>36</v>
       </c>
       <c r="E7" s="3" t="s">
@@ -1720,7 +2403,7 @@
       <c r="C8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E8" s="3" t="s">
@@ -1744,7 +2427,7 @@
       <c r="C9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="5" t="s">
         <v>24</v>
       </c>
       <c r="E9" s="3" t="s">
@@ -1768,7 +2451,7 @@
       <c r="C10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="8" t="s">
         <v>37</v>
       </c>
       <c r="E10" s="3" t="s">
@@ -1816,7 +2499,7 @@
       <c r="C12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E12" s="3" t="s">
@@ -1829,32 +2512,32 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="101.25" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
+    <row r="13" spans="1:7" ht="121.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="16">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" s="3" t="s">
+      <c r="B13" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="16" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="141.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="3">
+    <row r="14" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="17">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
@@ -1864,8 +2547,8 @@
       <c r="C14" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>18</v>
+      <c r="D14" s="17" t="s">
+        <v>40</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>6</v>
@@ -1877,8 +2560,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="81" x14ac:dyDescent="0.25">
-      <c r="A15" s="3">
+    <row r="15" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="17">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
@@ -1888,8 +2571,8 @@
       <c r="C15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>19</v>
+      <c r="D15" s="17" t="s">
+        <v>39</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>6</v>
@@ -1901,8 +2584,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="81" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
+    <row r="16" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="17">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
@@ -1912,8 +2595,8 @@
       <c r="C16" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>23</v>
+      <c r="D16" s="17" t="s">
+        <v>41</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>6</v>
@@ -1925,8 +2608,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="182.25" x14ac:dyDescent="0.25">
-      <c r="A17" s="3">
+    <row r="17" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="17">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
@@ -1936,8 +2619,8 @@
       <c r="C17" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>25</v>
+      <c r="D17" s="17" t="s">
+        <v>42</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>6</v>
@@ -1949,8 +2632,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="81" x14ac:dyDescent="0.25">
-      <c r="A18" s="3">
+    <row r="18" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="17">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
@@ -1960,8 +2643,8 @@
       <c r="C18" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>28</v>
+      <c r="D18" s="17" t="s">
+        <v>43</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>6</v>
@@ -1973,192 +2656,322 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="3">
-        <f t="shared" ref="A19:A21" si="1">A18+1</f>
+    <row r="19" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="17">
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="3">
-        <f t="shared" si="1"/>
+      <c r="C19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="17">
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="3">
-        <f t="shared" si="1"/>
+      <c r="C20" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="17">
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="3">
-        <f t="shared" ref="A22:A57" si="2">A21+1</f>
+      <c r="C21" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="17">
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="3">
-        <f t="shared" si="2"/>
+      <c r="C22" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="17">
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="3">
-        <f t="shared" si="2"/>
+      <c r="C23" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="17">
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="3">
-        <f t="shared" si="2"/>
+      <c r="C24" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="17">
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="3"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="3">
-        <f t="shared" si="2"/>
+      <c r="C25" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A26" s="17">
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="3">
-        <f t="shared" si="2"/>
+      <c r="C26" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="141.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="17">
+        <f>A23+1</f>
+        <v>22</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="81" x14ac:dyDescent="0.25">
+      <c r="A28" s="3">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="81" x14ac:dyDescent="0.25">
+      <c r="A29" s="3">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="182.25" x14ac:dyDescent="0.25">
+      <c r="A30" s="3">
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="B27" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="3">
-        <f t="shared" si="2"/>
+      <c r="B30" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="81" x14ac:dyDescent="0.25">
+      <c r="A31" s="3">
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="B28" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="3">
-        <f t="shared" si="2"/>
-        <v>27</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
-      <c r="G29" s="3"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="3">
-        <f t="shared" si="2"/>
+      <c r="B31" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
-      <c r="G30" s="3"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="3">
-        <f t="shared" si="2"/>
-        <v>29</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
+      <c r="E31" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
-        <f t="shared" si="2"/>
-        <v>30</v>
+        <f t="shared" ref="A32:A34" si="1">A31+1</f>
+        <v>27</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>13</v>
@@ -2171,8 +2984,8 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
-        <f t="shared" si="2"/>
-        <v>31</v>
+        <f t="shared" si="1"/>
+        <v>28</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>13</v>
@@ -2185,8 +2998,8 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
-        <f t="shared" si="2"/>
-        <v>32</v>
+        <f t="shared" si="1"/>
+        <v>29</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>13</v>
@@ -2199,8 +3012,8 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
-        <f t="shared" si="2"/>
-        <v>33</v>
+        <f t="shared" ref="A35:A70" si="2">A34+1</f>
+        <v>30</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>13</v>
@@ -2214,7 +3027,7 @@
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <f t="shared" si="2"/>
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>13</v>
@@ -2228,7 +3041,7 @@
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <f t="shared" si="2"/>
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>13</v>
@@ -2242,7 +3055,7 @@
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <f t="shared" si="2"/>
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>13</v>
@@ -2256,7 +3069,7 @@
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <f t="shared" si="2"/>
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>13</v>
@@ -2270,7 +3083,7 @@
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <f t="shared" si="2"/>
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>13</v>
@@ -2284,7 +3097,7 @@
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <f t="shared" si="2"/>
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>13</v>
@@ -2298,7 +3111,7 @@
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <f t="shared" si="2"/>
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>13</v>
@@ -2312,7 +3125,7 @@
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <f t="shared" si="2"/>
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>13</v>
@@ -2326,7 +3139,7 @@
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <f t="shared" si="2"/>
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>13</v>
@@ -2340,7 +3153,7 @@
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <f t="shared" si="2"/>
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>13</v>
@@ -2354,7 +3167,7 @@
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <f t="shared" si="2"/>
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>13</v>
@@ -2368,7 +3181,7 @@
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <f t="shared" si="2"/>
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>13</v>
@@ -2382,7 +3195,7 @@
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <f t="shared" si="2"/>
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>13</v>
@@ -2396,7 +3209,7 @@
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <f t="shared" si="2"/>
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>13</v>
@@ -2410,7 +3223,7 @@
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <f t="shared" si="2"/>
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>13</v>
@@ -2424,7 +3237,7 @@
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <f t="shared" si="2"/>
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>13</v>
@@ -2438,7 +3251,7 @@
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <f t="shared" si="2"/>
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>13</v>
@@ -2452,7 +3265,7 @@
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <f t="shared" si="2"/>
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>13</v>
@@ -2466,7 +3279,7 @@
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <f t="shared" si="2"/>
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>13</v>
@@ -2480,7 +3293,7 @@
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <f t="shared" si="2"/>
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>13</v>
@@ -2494,7 +3307,7 @@
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <f t="shared" si="2"/>
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>13</v>
@@ -2508,7 +3321,7 @@
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <f t="shared" si="2"/>
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>13</v>
@@ -2518,6 +3331,188 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" s="3">
+        <f t="shared" si="2"/>
+        <v>53</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C58" s="3"/>
+      <c r="D58" s="3"/>
+      <c r="E58" s="3"/>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" s="3">
+        <f t="shared" si="2"/>
+        <v>54</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C59" s="3"/>
+      <c r="D59" s="3"/>
+      <c r="E59" s="3"/>
+      <c r="F59" s="3"/>
+      <c r="G59" s="3"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" s="3">
+        <f t="shared" si="2"/>
+        <v>55</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C60" s="3"/>
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" s="3">
+        <f t="shared" si="2"/>
+        <v>56</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C61" s="3"/>
+      <c r="D61" s="3"/>
+      <c r="E61" s="3"/>
+      <c r="F61" s="3"/>
+      <c r="G61" s="3"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" s="3">
+        <f t="shared" si="2"/>
+        <v>57</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C62" s="3"/>
+      <c r="D62" s="3"/>
+      <c r="E62" s="3"/>
+      <c r="F62" s="3"/>
+      <c r="G62" s="3"/>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" s="3">
+        <f t="shared" si="2"/>
+        <v>58</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C63" s="3"/>
+      <c r="D63" s="3"/>
+      <c r="E63" s="3"/>
+      <c r="F63" s="3"/>
+      <c r="G63" s="3"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" s="3">
+        <f t="shared" si="2"/>
+        <v>59</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C64" s="3"/>
+      <c r="D64" s="3"/>
+      <c r="E64" s="3"/>
+      <c r="F64" s="3"/>
+      <c r="G64" s="3"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A65" s="3">
+        <f t="shared" si="2"/>
+        <v>60</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C65" s="3"/>
+      <c r="D65" s="3"/>
+      <c r="E65" s="3"/>
+      <c r="F65" s="3"/>
+      <c r="G65" s="3"/>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A66" s="3">
+        <f t="shared" si="2"/>
+        <v>61</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C66" s="3"/>
+      <c r="D66" s="3"/>
+      <c r="E66" s="3"/>
+      <c r="F66" s="3"/>
+      <c r="G66" s="3"/>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A67" s="3">
+        <f t="shared" si="2"/>
+        <v>62</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C67" s="3"/>
+      <c r="D67" s="3"/>
+      <c r="E67" s="3"/>
+      <c r="F67" s="3"/>
+      <c r="G67" s="3"/>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68" s="3">
+        <f t="shared" si="2"/>
+        <v>63</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C68" s="3"/>
+      <c r="D68" s="3"/>
+      <c r="E68" s="3"/>
+      <c r="F68" s="3"/>
+      <c r="G68" s="3"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A69" s="3">
+        <f t="shared" si="2"/>
+        <v>64</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C69" s="3"/>
+      <c r="D69" s="3"/>
+      <c r="E69" s="3"/>
+      <c r="F69" s="3"/>
+      <c r="G69" s="3"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A70" s="3">
+        <f t="shared" si="2"/>
+        <v>65</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C70" s="3"/>
+      <c r="D70" s="3"/>
+      <c r="E70" s="3"/>
+      <c r="F70" s="3"/>
+      <c r="G70" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2572,65 +3567,65 @@
       </c>
     </row>
     <row r="4" spans="1:3" ht="162" x14ac:dyDescent="0.25">
-      <c r="A4" s="5">
+      <c r="A4" s="4">
         <f>A3+1</f>
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="101.25" x14ac:dyDescent="0.25">
-      <c r="A5" s="5">
+      <c r="A5" s="4">
         <f>A4+1</f>
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="168" x14ac:dyDescent="0.25">
-      <c r="A6" s="5">
+      <c r="A6" s="4">
         <f>A5+1</f>
         <v>4</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
     </row>
     <row r="8" spans="1:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
     </row>
     <row r="9" spans="1:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
     </row>
     <row r="10" spans="1:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
     </row>
     <row r="11" spans="1:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
some more changes to the requirements list
</commit_message>
<xml_diff>
--- a/docs/spec/ARM.xlsx
+++ b/docs/spec/ARM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EitanKrimer\Documents\university\ADSS\ADSS_Group_Y\docs\spec\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBB33EFA-9F31-449B-B084-A44D2B0EBB48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFA440EB-89BC-47F9-B424-28900599CDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ARM" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="47">
   <si>
     <t>ID</t>
   </si>
@@ -58,9 +58,6 @@
   </si>
   <si>
     <t>MH</t>
-  </si>
-  <si>
-    <t>NTH</t>
   </si>
   <si>
     <t>High</t>
@@ -521,7 +518,57 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Upon maximum truck weight overflow - the system will ask the </t>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> can not allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="7" tint="-0.499984740745262"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>driver</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> without a sufficent drivers license type to drive any </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>truck</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">A </t>
     </r>
     <r>
       <rPr>
@@ -530,53 +577,16 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>TransportManager</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> which strategy to use:
-- </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="16"/>
-        <color rgb="FFE90505"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>cancel or change one of the destinations</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-- change truck
-- unload certain items from the current truck</t>
-    </r>
-  </si>
-  <si>
-    <t>Upon maximum truck weight overflow - the system will ask the TransportManager which strategy to use:
-- cancel or change one of the destinations
-- change truck
-- unload certain items from the current truck</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Don’t know what to do when
-"cancel or change one of the destinations" </t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The </t>
+      <t>Transport Manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> in The </t>
     </r>
     <r>
       <rPr>
@@ -594,74 +604,6 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> can not allow a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color theme="7" tint="-0.499984740745262"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>driver</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> without a sufficent drivers license type to drive any </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>truck</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">A </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Transport Manager</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> in The </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color theme="9" tint="-0.249977111117893"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>System</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
       <t xml:space="preserve"> can define a variaty of </t>
     </r>
     <r>
@@ -702,20 +644,6 @@
       </rPr>
       <t xml:space="preserve"> of the different Transports.</t>
     </r>
-  </si>
-  <si>
-    <t>NTH or MH?</t>
-  </si>
-  <si>
-    <t>How to alert?</t>
-  </si>
-  <si>
-    <t>בנוגע ל "אחראי ההובלה"
-מי הוא אחראי ההובלה מבחינתך?
-האם מדובר במשתמש מערכת שמחליט ברגע יצירת הובלה את ההתנהלות המועדפת בעת חריגה?</t>
-  </si>
-  <si>
-    <t>???</t>
   </si>
   <si>
     <r>
@@ -817,6 +745,752 @@
   </si>
   <si>
     <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to start a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to create a future </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to update a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to delete a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="5" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> a transport manager to create a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="7" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>driver</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to edit a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="7" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>driver</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to delete a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="7" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>driver</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to create a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>truck</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to edit a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>truck</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>transport manager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to delete a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>truck</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>admin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to create a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>branch</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>admin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to edit a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>branch</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>admin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to delete a </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>branch</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Upon maximum truck weight overflow - the system will ask the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>TransportManager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> which strategy to use:
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFE90505"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>cancel or change one of the destinations</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+- change truck
+- unload certain items from the current truck
+(Basically give the option to edit the entire transport)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>System</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> must allow an </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>admin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> to assign a user to the role of </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Transport Manager</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">For any Transport in the System, a Transport should have:
 - Transport ID
 - planned datetime of transport
@@ -916,9 +1590,14 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve"> ID(s) (FK)
+- completed sources - List of Site(s) ID(s)
+- completed destinations - List of Site(s) ID(s)
 - actual start datetime
 - actual end datetime</t>
     </r>
+  </si>
+  <si>
+    <t>The system must allow to check for requested items at supplier - if they exist - in which suppliers</t>
   </si>
   <si>
     <r>
@@ -946,658 +1625,9 @@
 - site object FK
 - contact phone
 - contact name
+- site address
 - OPTIONAL Delivery File ID ( FK to actual Delivery File)
-- OPTIONAL Recroded weight at site</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>System</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> must allow a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>transport manager</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> to start a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color theme="5" tint="-0.249977111117893"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>transport</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color theme="9" tint="-0.249977111117893"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>System</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> must allow a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>transport manager</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> to create a future </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color theme="5" tint="-0.249977111117893"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>transport</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>System</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> must allow a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>transport manager</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> to update a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color theme="5" tint="-0.249977111117893"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>transport</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>System</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> must allow a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>transport manager</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> to delete a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color theme="5" tint="-0.249977111117893"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>transport</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>System</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> must allow a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>transport manager</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> a transport manager to create a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color theme="7" tint="-0.249977111117893"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>driver</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>System</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> must allow a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>transport manager</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> to edit a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color theme="7" tint="-0.249977111117893"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>driver</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>System</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> must allow a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>transport manager</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> to delete a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color theme="7" tint="-0.249977111117893"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>driver</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>System</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> must allow a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>transport manager</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> to create a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>truck</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>System</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> must allow a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>transport manager</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> to edit a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>truck</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>System</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> must allow a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>transport manager</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> to delete a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>truck</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>System</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> must allow a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>admin</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> to create a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FFC00000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>branch</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>System</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> must allow a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>admin</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> to edit a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FFC00000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>branch</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>System</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> must allow a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>admin</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> to delete a </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <color rgb="FFC00000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>branch</t>
+- OPTIONAL Recorded weight at site</t>
     </r>
   </si>
 </sst>
@@ -1781,18 +1811,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1891,7 +1915,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
@@ -1911,11 +1935,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -1937,12 +1961,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2232,7 +2250,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="21" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
@@ -2253,7 +2271,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D1" s="9" t="s">
         <v>2</v>
@@ -2282,18 +2300,22 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="101.25" x14ac:dyDescent="0.25">
@@ -2302,22 +2324,22 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="D4" s="5" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="162" x14ac:dyDescent="0.25">
@@ -2326,46 +2348,46 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="D5" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="141.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
-        <f t="shared" ref="A6:A31" si="0">A5+1</f>
+        <f t="shared" ref="A6:A33" si="0">A5+1</f>
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="D6" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="141.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2374,46 +2396,46 @@
         <v>5</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="D7" s="5" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="222.75" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="243" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="D8" s="5" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="140.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2422,46 +2444,46 @@
         <v>7</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="D9" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="342" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>37</v>
+      <c r="D10" s="7" t="s">
+        <v>44</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
@@ -2470,22 +2492,22 @@
         <v>9</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="D11" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="101.25" x14ac:dyDescent="0.25">
@@ -2494,454 +2516,454 @@
         <v>10</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="D12" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="121.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="16">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="81" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="B13" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="D13" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" s="16" t="s">
+      <c r="B13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F13" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="G13" s="16" t="s">
+      <c r="G13" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="8" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="17">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D14" s="17" t="s">
-        <v>40</v>
+      <c r="D14" s="3" t="s">
+        <v>43</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="17">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="121.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D15" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="E15" s="3" t="s">
+      <c r="B15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E15" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>15</v>
+      <c r="F15" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="17">
+      <c r="A16" s="8">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D16" s="17" t="s">
-        <v>41</v>
+        <v>15</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>30</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="17">
+      <c r="A17" s="8">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D17" s="17" t="s">
-        <v>42</v>
+        <v>15</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="17">
+      <c r="A18" s="8">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D18" s="17" t="s">
-        <v>43</v>
+        <v>15</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>31</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="17">
+      <c r="A19" s="8">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D19" s="17" t="s">
-        <v>44</v>
+        <v>15</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>32</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="17">
+      <c r="A20" s="8">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D20" s="17" t="s">
-        <v>45</v>
+        <v>15</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>33</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="17">
+      <c r="A21" s="8">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D21" s="17" t="s">
-        <v>46</v>
+        <v>15</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>34</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="17">
+      <c r="A22" s="8">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D22" s="17" t="s">
-        <v>47</v>
+        <v>15</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>35</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="17">
+      <c r="A23" s="8">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D23" s="17" t="s">
-        <v>48</v>
+        <v>15</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>36</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="17">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="8">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D24" s="17" t="s">
-        <v>49</v>
+        <v>15</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>37</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
-      <c r="A25" s="17">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="8">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D25" s="17" t="s">
-        <v>50</v>
+        <v>15</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
-      <c r="A26" s="17">
+      <c r="A26" s="8">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D26" s="17" t="s">
-        <v>51</v>
+        <v>15</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>39</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G26" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A27" s="8">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" ht="141.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="17">
-        <f>A23+1</f>
-        <v>22</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>18</v>
+      <c r="D27" s="8" t="s">
+        <v>40</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G27" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="8">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" ht="81" x14ac:dyDescent="0.25">
-      <c r="A28" s="3">
-        <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>19</v>
+      <c r="D28" s="8" t="s">
+        <v>41</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G28" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="141.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="8">
+        <f>A25+1</f>
+        <v>24</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C29" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" ht="81" x14ac:dyDescent="0.25">
-      <c r="A29" s="3">
-        <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="D29" s="3" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="182.25" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="81" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="81" x14ac:dyDescent="0.25">
@@ -2950,59 +2972,79 @@
         <v>26</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>6</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G31" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="222.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="3">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="3">
-        <f t="shared" ref="A32:A34" si="1">A31+1</f>
-        <v>27</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D32" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="81" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
+        <v>12</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="A34:A36" si="1">A33+1</f>
         <v>29</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
@@ -3012,11 +3054,11 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
-        <f t="shared" ref="A35:A70" si="2">A34+1</f>
+        <f t="shared" si="1"/>
         <v>30</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
@@ -3026,11 +3068,11 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>31</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
@@ -3040,11 +3082,11 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="A37:A72" si="2">A36+1</f>
         <v>32</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
@@ -3058,7 +3100,7 @@
         <v>33</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
@@ -3072,7 +3114,7 @@
         <v>34</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
@@ -3086,7 +3128,7 @@
         <v>35</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
@@ -3100,7 +3142,7 @@
         <v>36</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
@@ -3114,7 +3156,7 @@
         <v>37</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
@@ -3128,7 +3170,7 @@
         <v>38</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
@@ -3142,7 +3184,7 @@
         <v>39</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
@@ -3156,7 +3198,7 @@
         <v>40</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
@@ -3170,7 +3212,7 @@
         <v>41</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
@@ -3184,7 +3226,7 @@
         <v>42</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
@@ -3198,7 +3240,7 @@
         <v>43</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
@@ -3212,7 +3254,7 @@
         <v>44</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
@@ -3226,7 +3268,7 @@
         <v>45</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
@@ -3240,7 +3282,7 @@
         <v>46</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
@@ -3254,7 +3296,7 @@
         <v>47</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
@@ -3268,7 +3310,7 @@
         <v>48</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
@@ -3282,7 +3324,7 @@
         <v>49</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
@@ -3296,7 +3338,7 @@
         <v>50</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
@@ -3310,7 +3352,7 @@
         <v>51</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C56" s="3"/>
       <c r="D56" s="3"/>
@@ -3324,7 +3366,7 @@
         <v>52</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C57" s="3"/>
       <c r="D57" s="3"/>
@@ -3338,7 +3380,7 @@
         <v>53</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
@@ -3352,7 +3394,7 @@
         <v>54</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
@@ -3366,7 +3408,7 @@
         <v>55</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C60" s="3"/>
       <c r="D60" s="3"/>
@@ -3380,7 +3422,7 @@
         <v>56</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C61" s="3"/>
       <c r="D61" s="3"/>
@@ -3394,7 +3436,7 @@
         <v>57</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C62" s="3"/>
       <c r="D62" s="3"/>
@@ -3408,7 +3450,7 @@
         <v>58</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C63" s="3"/>
       <c r="D63" s="3"/>
@@ -3422,7 +3464,7 @@
         <v>59</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C64" s="3"/>
       <c r="D64" s="3"/>
@@ -3436,7 +3478,7 @@
         <v>60</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C65" s="3"/>
       <c r="D65" s="3"/>
@@ -3450,7 +3492,7 @@
         <v>61</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C66" s="3"/>
       <c r="D66" s="3"/>
@@ -3464,7 +3506,7 @@
         <v>62</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C67" s="3"/>
       <c r="D67" s="3"/>
@@ -3478,7 +3520,7 @@
         <v>63</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C68" s="3"/>
       <c r="D68" s="3"/>
@@ -3492,7 +3534,7 @@
         <v>64</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C69" s="3"/>
       <c r="D69" s="3"/>
@@ -3506,13 +3548,41 @@
         <v>65</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C70" s="3"/>
       <c r="D70" s="3"/>
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
       <c r="G70" s="3"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" s="3">
+        <f t="shared" si="2"/>
+        <v>66</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C71" s="3"/>
+      <c r="D71" s="3"/>
+      <c r="E71" s="3"/>
+      <c r="F71" s="3"/>
+      <c r="G71" s="3"/>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A72" s="3">
+        <f t="shared" si="2"/>
+        <v>67</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C72" s="3"/>
+      <c r="D72" s="3"/>
+      <c r="E72" s="3"/>
+      <c r="F72" s="3"/>
+      <c r="G72" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -3539,7 +3609,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="15"/>
@@ -3549,58 +3619,42 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="135" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="162" x14ac:dyDescent="0.25">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+    </row>
+    <row r="4" spans="1:3" ht="21" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <f>A3+1</f>
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="101.25" x14ac:dyDescent="0.25">
+      <c r="B4" s="3"/>
+      <c r="C4" s="4"/>
+    </row>
+    <row r="5" spans="1:3" ht="21" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <f>A4+1</f>
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="168" x14ac:dyDescent="0.25">
+      <c r="B5" s="3"/>
+      <c r="C5" s="4"/>
+    </row>
+    <row r="6" spans="1:3" ht="21" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <f>A5+1</f>
         <v>4</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>33</v>
-      </c>
+      <c r="B6" s="6"/>
+      <c r="C6" s="4"/>
     </row>
     <row r="7" spans="1:3" ht="21" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>

</xml_diff>

<commit_message>
Edit docu and release
</commit_message>
<xml_diff>
--- a/docs/spec/ARM.xlsx
+++ b/docs/spec/ARM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\taoma\Downloads\תיכון ותכנון מערכות\ADSS_Group_Y\docs\spec\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EitanKrimer\Documents\university\ADSS\ADSS_Group_Y\docs\spec\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C4554CB-FC66-4CC4-96B3-7AE9CB56AE0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAAB8A9D-C85D-46D8-8A5D-2F6A409DCB27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="1800" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ARM" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="81">
   <si>
     <t>ID</t>
   </si>
@@ -601,9 +601,6 @@
 - Unloaded Items Delivery File ID
 - Transport route ID </t>
     </r>
-  </si>
-  <si>
-    <t>הגעתי עד פה</t>
   </si>
   <si>
     <r>
@@ -2581,7 +2578,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -2600,7 +2597,7 @@
     <font>
       <sz val="16"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -2807,7 +2804,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2817,12 +2814,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2943,11 +2934,14 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -2961,9 +2955,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="20" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -2973,8 +2964,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3265,51 +3256,51 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H76"/>
-  <sheetFormatPr defaultColWidth="9.09765625" defaultRowHeight="20.399999999999999" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="21" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.09765625" style="2"/>
-    <col min="2" max="2" width="15.3984375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="2"/>
+    <col min="2" max="2" width="15.42578125" style="2" customWidth="1"/>
     <col min="3" max="3" width="10" style="2" customWidth="1"/>
-    <col min="4" max="4" width="43.59765625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="12.09765625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.09765625" style="2"/>
-    <col min="7" max="7" width="26.296875" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="9.09765625" style="2"/>
+    <col min="4" max="4" width="43.5703125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" style="2"/>
+    <col min="7" max="7" width="26.28515625" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="12" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-    </row>
-    <row r="3" spans="1:7" ht="123" x14ac:dyDescent="0.25">
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+    </row>
+    <row r="3" spans="1:7" ht="121.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -3332,7 +3323,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="102.6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="101.25" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <f>A3+1</f>
         <v>2</v>
@@ -3356,7 +3347,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="163.19999999999999" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="162" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <f>A4+1</f>
         <v>3</v>
@@ -3404,7 +3395,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="178.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="178.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -3452,7 +3443,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="226.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="226.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -3476,7 +3467,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="343.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="343.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <f>A9+1</f>
         <v>8</v>
@@ -3488,7 +3479,7 @@
         <v>13</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>6</v>
@@ -3500,7 +3491,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="142.19999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="142.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -3511,19 +3502,19 @@
         <v>13</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="9" t="s">
         <v>7</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -3546,7 +3537,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="102" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="101.25" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -3558,7 +3549,7 @@
         <v>13</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>6</v>
@@ -3570,7 +3561,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="81" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -3585,16 +3576,16 @@
         <v>24</v>
       </c>
       <c r="E14" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F14" s="3" t="s">
-        <v>33</v>
-      </c>
       <c r="G14" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -3609,16 +3600,16 @@
         <v>23</v>
       </c>
       <c r="E15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="3" t="s">
-        <v>33</v>
-      </c>
       <c r="G15" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="64.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8">
         <v>14</v>
       </c>
@@ -3629,10 +3620,10 @@
         <v>15</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>7</v>
@@ -3641,7 +3632,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="64.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="64.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8">
         <v>15</v>
       </c>
@@ -3652,10 +3643,10 @@
         <v>15</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>7</v>
@@ -3664,7 +3655,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A18" s="8">
         <v>16</v>
       </c>
@@ -3675,7 +3666,7 @@
         <v>15</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>6</v>
@@ -3687,7 +3678,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A19" s="8">
         <v>17</v>
       </c>
@@ -3698,7 +3689,7 @@
         <v>15</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>6</v>
@@ -3710,7 +3701,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A20" s="8">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -3722,7 +3713,7 @@
         <v>15</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>6</v>
@@ -3734,7 +3725,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="81.599999999999994" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="81" x14ac:dyDescent="0.25">
       <c r="A21" s="8">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -3746,7 +3737,7 @@
         <v>15</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>6</v>
@@ -3758,7 +3749,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A22" s="8">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -3770,7 +3761,7 @@
         <v>15</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>6</v>
@@ -3782,7 +3773,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A23" s="8">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -3794,7 +3785,7 @@
         <v>15</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>6</v>
@@ -3806,7 +3797,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A24" s="8">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -3818,7 +3809,7 @@
         <v>15</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>6</v>
@@ -3830,7 +3821,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A25" s="8">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -3842,7 +3833,7 @@
         <v>15</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>6</v>
@@ -3854,7 +3845,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A26" s="8">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -3866,7 +3857,7 @@
         <v>15</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>6</v>
@@ -3878,7 +3869,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A27" s="8">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -3890,7 +3881,7 @@
         <v>15</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>6</v>
@@ -3902,7 +3893,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A28" s="8">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -3914,7 +3905,7 @@
         <v>15</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>6</v>
@@ -3926,7 +3917,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A29" s="8">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -3938,7 +3929,7 @@
         <v>15</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>6</v>
@@ -3950,7 +3941,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A30" s="8">
         <v>29</v>
       </c>
@@ -3961,7 +3952,7 @@
         <v>15</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>6</v>
@@ -3973,7 +3964,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A31" s="8">
         <v>30</v>
       </c>
@@ -3984,7 +3975,7 @@
         <v>15</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>6</v>
@@ -3996,7 +3987,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A32" s="8">
         <v>31</v>
       </c>
@@ -4007,7 +3998,7 @@
         <v>15</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>6</v>
@@ -4019,7 +4010,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="142.80000000000001" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="141.75" x14ac:dyDescent="0.25">
       <c r="A33" s="8">
         <v>32</v>
       </c>
@@ -4033,7 +4024,7 @@
         <v>17</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>7</v>
@@ -4042,7 +4033,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="122.4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="121.5" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <f t="shared" si="0"/>
         <v>33</v>
@@ -4054,10 +4045,10 @@
         <v>15</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>7</v>
@@ -4066,7 +4057,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="81" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -4084,13 +4075,13 @@
         <v>6</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="225.6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="222.75" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -4102,7 +4093,7 @@
         <v>15</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>6</v>
@@ -4114,7 +4105,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="81" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <f t="shared" si="0"/>
         <v>36</v>
@@ -4138,7 +4129,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <f t="shared" ref="A38:A40" si="1">A37+1</f>
         <v>37</v>
@@ -4150,7 +4141,7 @@
         <v>15</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>6</v>
@@ -4162,7 +4153,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <f t="shared" si="1"/>
         <v>38</v>
@@ -4174,7 +4165,7 @@
         <v>15</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>6</v>
@@ -4186,7 +4177,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <f t="shared" si="1"/>
         <v>39</v>
@@ -4198,7 +4189,7 @@
         <v>15</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>6</v>
@@ -4210,7 +4201,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <f t="shared" ref="A41:A76" si="2">A40+1</f>
         <v>40</v>
@@ -4222,7 +4213,7 @@
         <v>15</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>6</v>
@@ -4234,7 +4225,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <f t="shared" si="2"/>
         <v>41</v>
@@ -4246,19 +4237,19 @@
         <v>15</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F42" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F42" s="10" t="s">
         <v>7</v>
       </c>
       <c r="G42" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <f t="shared" si="2"/>
         <v>42</v>
@@ -4270,10 +4261,10 @@
         <v>15</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>7</v>
@@ -4281,11 +4272,9 @@
       <c r="G43" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H43" s="9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" ht="61.2" x14ac:dyDescent="0.25">
+      <c r="H43" s="19"/>
+    </row>
+    <row r="44" spans="1:8" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <f t="shared" si="2"/>
         <v>43</v>
@@ -4297,10 +4286,10 @@
         <v>15</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>7</v>
@@ -4309,7 +4298,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <f t="shared" si="2"/>
         <v>44</v>
@@ -4321,10 +4310,10 @@
         <v>15</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F45" s="3" t="s">
         <v>7</v>
@@ -4333,7 +4322,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="61.2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" ht="60.75" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <f t="shared" si="2"/>
         <v>45</v>
@@ -4345,10 +4334,10 @@
         <v>15</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>7</v>
@@ -4357,7 +4346,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <f t="shared" si="2"/>
         <v>46</v>
@@ -4369,7 +4358,7 @@
         <v>15</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E47" s="3" t="s">
         <v>6</v>
@@ -4381,7 +4370,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <f t="shared" si="2"/>
         <v>47</v>
@@ -4393,7 +4382,7 @@
         <v>15</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>6</v>
@@ -4405,7 +4394,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <f t="shared" si="2"/>
         <v>48</v>
@@ -4417,7 +4406,7 @@
         <v>15</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>6</v>
@@ -4429,7 +4418,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <f t="shared" si="2"/>
         <v>49</v>
@@ -4441,7 +4430,7 @@
         <v>15</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>6</v>
@@ -4453,7 +4442,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <f t="shared" si="2"/>
         <v>50</v>
@@ -4465,7 +4454,7 @@
         <v>15</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>6</v>
@@ -4477,7 +4466,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <f t="shared" si="2"/>
         <v>51</v>
@@ -4489,7 +4478,7 @@
         <v>15</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>6</v>
@@ -4501,7 +4490,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <f t="shared" si="2"/>
         <v>52</v>
@@ -4510,10 +4499,10 @@
         <v>12</v>
       </c>
       <c r="C53" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D53" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="D53" s="3" t="s">
-        <v>70</v>
       </c>
       <c r="E53" s="3" t="s">
         <v>6</v>
@@ -4525,7 +4514,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="61.8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="81" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <f t="shared" si="2"/>
         <v>53</v>
@@ -4537,7 +4526,7 @@
         <v>13</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E54" s="3" t="s">
         <v>6</v>
@@ -4875,21 +4864,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6A548FC-132A-4BCF-B26C-A9E84109E40A}">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="34.69921875" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="20.399999999999999" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
         <v>11</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="18"/>
-      <c r="D1" s="19"/>
-    </row>
-    <row r="2" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="D1" s="11"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -4899,62 +4888,62 @@
       <c r="C2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="19"/>
+      <c r="D2" s="11"/>
     </row>
     <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D3" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D3" s="19" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="40.799999999999997" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:4" ht="42" x14ac:dyDescent="0.25">
       <c r="A4" s="6">
         <f>A3+1</f>
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="D4" s="19"/>
-    </row>
-    <row r="5" spans="1:4" ht="61.2" x14ac:dyDescent="0.25">
+      <c r="D4" s="11"/>
+    </row>
+    <row r="5" spans="1:4" ht="63" x14ac:dyDescent="0.25">
       <c r="A5" s="6">
         <f>A4+1</f>
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="D5" s="19"/>
-    </row>
-    <row r="6" spans="1:4" ht="61.2" x14ac:dyDescent="0.25">
+      <c r="D5" s="11"/>
+    </row>
+    <row r="6" spans="1:4" ht="63" x14ac:dyDescent="0.25">
       <c r="A6" s="6">
         <f>A5+1</f>
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="D6" s="19"/>
-    </row>
-    <row r="7" spans="1:4" ht="40.799999999999997" x14ac:dyDescent="0.25">
+      <c r="D6" s="11"/>
+    </row>
+    <row r="7" spans="1:4" ht="42" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>5</v>
       </c>
@@ -4962,25 +4951,25 @@
         <v>12</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="20.399999999999999" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="21" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
     </row>
-    <row r="9" spans="1:4" ht="20.399999999999999" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ht="21" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
     </row>
-    <row r="10" spans="1:4" ht="20.399999999999999" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="21" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
     </row>
-    <row r="11" spans="1:4" ht="20.399999999999999" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="21" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>

</xml_diff>